<commit_message>
extend categoria labels: LECERs and BONTE coupon bonds
Per user request:
  - 5 LECERs (X15Y6, X29Y6, X31L6, X30S6, X30N6) -> "LETRA TESORO DESCUENTO CER"
  - DICP, CUAP, PARP (all freq=2 semestral) -> "BONTE (SEMESTRAL)"

DIPO and PAPO left blank (user did not include them; they are peso-dollar
variants of the same family).

All 21 live CER bonds now have a populated categoria field.
</commit_message>
<xml_diff>
--- a/data/instruments_master.xlsx
+++ b/data/instruments_master.xlsx
@@ -1618,6 +1618,11 @@
       <c r="M2" t="n">
         <v>701.61402891428</v>
       </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>LETRA TESORO DESCUENTO CER</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1642,6 +1647,11 @@
       <c r="M3" t="n">
         <v>652.33524435885</v>
       </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>LETRA TESORO DESCUENTO CER</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1695,6 +1705,11 @@
       <c r="M5" t="n">
         <v>685.55061207521</v>
       </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>LETRA TESORO DESCUENTO CER</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1719,6 +1734,11 @@
       <c r="M6" t="n">
         <v>714.9848780192</v>
       </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>LETRA TESORO DESCUENTO CER</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1823,6 +1843,11 @@
       <c r="M9" t="n">
         <v>659.67889566652</v>
       </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>LETRA TESORO DESCUENTO CER</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2145,6 +2170,11 @@
       <c r="M18" t="n">
         <v>1.4550639398</v>
       </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>BONTE (SEMESTRAL)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2198,6 +2228,11 @@
       <c r="M19" t="n">
         <v>1.4550639398</v>
       </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>BONTE (SEMESTRAL)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2243,6 +2278,11 @@
       </c>
       <c r="M20" t="n">
         <v>1.4550639398</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>BONTE (SEMESTRAL)</t>
+        </is>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Flujo y clalendario de pagos ONs
</commit_message>
<xml_diff>
--- a/data/instruments_master.xlsx
+++ b/data/instruments_master.xlsx
@@ -14424,7 +14424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R262"/>
+  <dimension ref="A1:R260"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22305,7 +22305,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>TLCLD</t>
+          <t>TLCUD</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -22330,20 +22330,20 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>AR0731472459</t>
+          <t>AR0857544677</t>
         </is>
       </c>
       <c r="G129" s="25" t="n">
-        <v>45449</v>
+        <v>46086</v>
       </c>
       <c r="H129" s="25" t="n">
-        <v>46179</v>
+        <v>47182</v>
       </c>
       <c r="I129" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="J129" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K129" t="inlineStr">
         <is>
@@ -22356,16 +22356,19 @@
         </is>
       </c>
       <c r="M129" s="25" t="n">
-        <v>46179</v>
+        <v>47182</v>
       </c>
       <c r="N129" t="n">
         <v>1</v>
       </c>
+      <c r="O129" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>TLCUD</t>
+          <t>TLCDD</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -22390,20 +22393,20 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>AR0857544677</t>
+          <t>ARTECO5600E0</t>
         </is>
       </c>
       <c r="G130" s="25" t="n">
-        <v>46086</v>
+        <v>44629</v>
       </c>
       <c r="H130" s="25" t="n">
-        <v>47182</v>
+        <v>46455</v>
       </c>
       <c r="I130" t="n">
-        <v>6.5</v>
+        <v>1</v>
       </c>
       <c r="J130" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K130" t="inlineStr">
         <is>
@@ -22416,24 +22419,21 @@
         </is>
       </c>
       <c r="M130" s="25" t="n">
-        <v>47182</v>
+        <v>46455</v>
       </c>
       <c r="N130" t="n">
         <v>1</v>
       </c>
-      <c r="O130" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>TLCDD</t>
+          <t>VSCQD</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>Vista Energy</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -22443,7 +22443,7 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Telecomunicaciones</t>
+          <t>Petróleo y Gas</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
@@ -22453,17 +22453,17 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>ARTECO5600E0</t>
+          <t>AR0941463967</t>
         </is>
       </c>
       <c r="G131" s="25" t="n">
-        <v>44629</v>
+        <v>45481</v>
       </c>
       <c r="H131" s="25" t="n">
-        <v>46455</v>
+        <v>46942</v>
       </c>
       <c r="I131" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J131" t="n">
         <v>4</v>
@@ -22479,7 +22479,7 @@
         </is>
       </c>
       <c r="M131" s="25" t="n">
-        <v>46455</v>
+        <v>46942</v>
       </c>
       <c r="N131" t="n">
         <v>1</v>
@@ -22488,7 +22488,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>VSCQD</t>
+          <t>VSCMD</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -22513,17 +22513,17 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>AR0941463967</t>
+          <t>AROILG5600L4</t>
         </is>
       </c>
       <c r="G132" s="25" t="n">
-        <v>45481</v>
+        <v>45149</v>
       </c>
       <c r="H132" s="25" t="n">
-        <v>46942</v>
+        <v>46976</v>
       </c>
       <c r="I132" t="n">
-        <v>3</v>
+        <v>0.99</v>
       </c>
       <c r="J132" t="n">
         <v>4</v>
@@ -22539,7 +22539,7 @@
         </is>
       </c>
       <c r="M132" s="25" t="n">
-        <v>46942</v>
+        <v>46976</v>
       </c>
       <c r="N132" t="n">
         <v>1</v>
@@ -22548,7 +22548,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>VSCMD</t>
+          <t>VSCWD</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -22573,17 +22573,17 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t>AROILG5600L4</t>
+          <t>AR0652555118</t>
         </is>
       </c>
       <c r="G133" s="25" t="n">
-        <v>45149</v>
+        <v>45945</v>
       </c>
       <c r="H133" s="25" t="n">
-        <v>46976</v>
+        <v>46492</v>
       </c>
       <c r="I133" t="n">
-        <v>0.99</v>
+        <v>6</v>
       </c>
       <c r="J133" t="n">
         <v>4</v>
@@ -22599,7 +22599,7 @@
         </is>
       </c>
       <c r="M133" s="25" t="n">
-        <v>46976</v>
+        <v>46492</v>
       </c>
       <c r="N133" t="n">
         <v>1</v>
@@ -22608,7 +22608,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>VSCWD</t>
+          <t>VSCOD</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -22633,20 +22633,20 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>AR0652555118</t>
+          <t>AR0399155156</t>
         </is>
       </c>
       <c r="G134" s="25" t="n">
-        <v>45945</v>
+        <v>45357</v>
       </c>
       <c r="H134" s="25" t="n">
-        <v>46492</v>
+        <v>46452</v>
       </c>
       <c r="I134" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="J134" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K134" t="inlineStr">
         <is>
@@ -22659,7 +22659,7 @@
         </is>
       </c>
       <c r="M134" s="25" t="n">
-        <v>46492</v>
+        <v>46452</v>
       </c>
       <c r="N134" t="n">
         <v>1</v>
@@ -22668,7 +22668,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>VSCOD</t>
+          <t>VSCUD</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -22693,17 +22693,17 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>AR0399155156</t>
+          <t>AR0707929003</t>
         </is>
       </c>
       <c r="G135" s="25" t="n">
-        <v>45357</v>
+        <v>45723</v>
       </c>
       <c r="H135" s="25" t="n">
-        <v>46452</v>
+        <v>47549</v>
       </c>
       <c r="I135" t="n">
-        <v>6.5</v>
+        <v>7.5</v>
       </c>
       <c r="J135" t="n">
         <v>2</v>
@@ -22719,7 +22719,7 @@
         </is>
       </c>
       <c r="M135" s="25" t="n">
-        <v>46452</v>
+        <v>47549</v>
       </c>
       <c r="N135" t="n">
         <v>1</v>
@@ -22728,7 +22728,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>VSCUD</t>
+          <t>VSCJD</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -22753,20 +22753,20 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>AR0707929003</t>
+          <t>AROILG5600I0</t>
         </is>
       </c>
       <c r="G136" s="25" t="n">
-        <v>45723</v>
+        <v>44988</v>
       </c>
       <c r="H136" s="25" t="n">
-        <v>47549</v>
+        <v>46449</v>
       </c>
       <c r="I136" t="n">
-        <v>7.5</v>
+        <v>0</v>
       </c>
       <c r="J136" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K136" t="inlineStr">
         <is>
@@ -22779,7 +22779,7 @@
         </is>
       </c>
       <c r="M136" s="25" t="n">
-        <v>47549</v>
+        <v>46449</v>
       </c>
       <c r="N136" t="n">
         <v>1</v>
@@ -22788,7 +22788,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>VSCHD</t>
+          <t>VSCRD</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -22813,20 +22813,20 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>AROILG5600G4</t>
+          <t>AR0138120560</t>
         </is>
       </c>
       <c r="G137" s="25" t="n">
-        <v>44901</v>
+        <v>45575</v>
       </c>
       <c r="H137" s="25" t="n">
-        <v>46179</v>
+        <v>48131</v>
       </c>
       <c r="I137" t="n">
-        <v>0</v>
+        <v>7.65</v>
       </c>
       <c r="J137" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K137" t="inlineStr">
         <is>
@@ -22835,25 +22835,31 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>bullet</t>
+          <t>amortizing</t>
         </is>
       </c>
       <c r="M137" s="25" t="n">
-        <v>46179</v>
+        <v>47401</v>
       </c>
       <c r="N137" t="n">
+        <v>3</v>
+      </c>
+      <c r="O137" t="n">
         <v>1</v>
+      </c>
+      <c r="P137" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>VSCJD</t>
+          <t>YFCLD</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Vista Energy</t>
+          <t>YPF Energia Electrica SA</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -22863,7 +22869,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Petróleo y Gas</t>
+          <t>Servicios Públicos y Generación</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
@@ -22873,24 +22879,24 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>AROILG5600I0</t>
+          <t>AR0338531962</t>
         </is>
       </c>
       <c r="G138" s="25" t="n">
-        <v>44988</v>
+        <v>45618</v>
       </c>
       <c r="H138" s="25" t="n">
-        <v>46449</v>
+        <v>47079</v>
       </c>
       <c r="I138" t="n">
-        <v>0</v>
+        <v>6.75</v>
       </c>
       <c r="J138" t="n">
         <v>4</v>
       </c>
       <c r="K138" t="inlineStr">
         <is>
-          <t>ACT/365</t>
+          <t>30/360</t>
         </is>
       </c>
       <c r="L138" t="inlineStr">
@@ -22899,7 +22905,7 @@
         </is>
       </c>
       <c r="M138" s="25" t="n">
-        <v>46449</v>
+        <v>47079</v>
       </c>
       <c r="N138" t="n">
         <v>1</v>
@@ -22908,12 +22914,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>VSCRD</t>
+          <t>YFCMD</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Vista Energy</t>
+          <t>YPF Energia Electrica SA</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -22923,7 +22929,7 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Petróleo y Gas</t>
+          <t>Servicios Públicos y Generación</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -22933,48 +22939,42 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>AR0138120560</t>
+          <t>AR0975634988</t>
         </is>
       </c>
       <c r="G139" s="25" t="n">
-        <v>45575</v>
+        <v>45797</v>
       </c>
       <c r="H139" s="25" t="n">
-        <v>48131</v>
+        <v>46527</v>
       </c>
       <c r="I139" t="n">
-        <v>7.65</v>
+        <v>6.5</v>
       </c>
       <c r="J139" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>ACT/365</t>
+          <t>30/360</t>
         </is>
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>amortizing</t>
+          <t>bullet</t>
         </is>
       </c>
       <c r="M139" s="25" t="n">
-        <v>47401</v>
+        <v>46527</v>
       </c>
       <c r="N139" t="n">
-        <v>3</v>
-      </c>
-      <c r="O139" t="n">
         <v>1</v>
-      </c>
-      <c r="P139" t="n">
-        <v>33</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>YFCLD</t>
+          <t>YFCAD</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -22999,20 +22999,20 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>AR0338531962</t>
+          <t>ARYPFE5600G5</t>
         </is>
       </c>
       <c r="G140" s="25" t="n">
-        <v>45618</v>
+        <v>44595</v>
       </c>
       <c r="H140" s="25" t="n">
-        <v>47079</v>
+        <v>48247</v>
       </c>
       <c r="I140" t="n">
-        <v>6.75</v>
+        <v>5</v>
       </c>
       <c r="J140" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K140" t="inlineStr">
         <is>
@@ -23021,20 +23021,26 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>bullet</t>
+          <t>amortizing</t>
         </is>
       </c>
       <c r="M140" s="25" t="n">
-        <v>47079</v>
+        <v>46602</v>
       </c>
       <c r="N140" t="n">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="O140" t="n">
+        <v>2</v>
+      </c>
+      <c r="P140" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>YFCMD</t>
+          <t>YFCND</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -23059,20 +23065,20 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>AR0975634988</t>
+          <t>AR0361875989</t>
         </is>
       </c>
       <c r="G141" s="25" t="n">
-        <v>45797</v>
+        <v>45933</v>
       </c>
       <c r="H141" s="25" t="n">
-        <v>46527</v>
+        <v>46298</v>
       </c>
       <c r="I141" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="J141" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K141" t="inlineStr">
         <is>
@@ -23085,7 +23091,7 @@
         </is>
       </c>
       <c r="M141" s="25" t="n">
-        <v>46527</v>
+        <v>46298</v>
       </c>
       <c r="N141" t="n">
         <v>1</v>
@@ -23094,12 +23100,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>YFCAD</t>
+          <t>YM40D</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>YPF Energia Electrica SA</t>
+          <t>YPF SA</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -23109,7 +23115,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Servicios Públicos y Generación</t>
+          <t>Petróleo y Gas</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -23119,53 +23125,47 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>ARYPFE5600G5</t>
+          <t>AR0963751125</t>
         </is>
       </c>
       <c r="G142" s="25" t="n">
-        <v>44595</v>
+        <v>45897</v>
       </c>
       <c r="H142" s="25" t="n">
-        <v>48247</v>
+        <v>46993</v>
       </c>
       <c r="I142" t="n">
-        <v>5</v>
+        <v>7.5</v>
       </c>
       <c r="J142" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>30/360</t>
+          <t>ACT/365</t>
         </is>
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>amortizing</t>
+          <t>bullet</t>
         </is>
       </c>
       <c r="M142" s="25" t="n">
-        <v>46602</v>
+        <v>46993</v>
       </c>
       <c r="N142" t="n">
-        <v>10</v>
-      </c>
-      <c r="O142" t="n">
-        <v>2</v>
-      </c>
-      <c r="P142" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>YFCND</t>
+          <t>YM41D</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>YPF Energia Electrica SA</t>
+          <t>YPF SA</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -23175,7 +23175,7 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Servicios Públicos y Generación</t>
+          <t>Petróleo y Gas</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -23185,24 +23185,24 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>AR0361875989</t>
+          <t>AR0675705039</t>
         </is>
       </c>
       <c r="G143" s="25" t="n">
-        <v>45933</v>
+        <v>45938</v>
       </c>
       <c r="H143" s="25" t="n">
-        <v>46298</v>
+        <v>46395</v>
       </c>
       <c r="I143" t="n">
         <v>6</v>
       </c>
       <c r="J143" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>30/360</t>
+          <t>ACT/365</t>
         </is>
       </c>
       <c r="L143" t="inlineStr">
@@ -23211,7 +23211,7 @@
         </is>
       </c>
       <c r="M143" s="25" t="n">
-        <v>46298</v>
+        <v>46395</v>
       </c>
       <c r="N143" t="n">
         <v>1</v>
@@ -23220,7 +23220,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>YM40D</t>
+          <t>YMCYD</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -23245,17 +23245,17 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t>AR0963751125</t>
+          <t>AR0417757066</t>
         </is>
       </c>
       <c r="G144" s="25" t="n">
-        <v>45897</v>
+        <v>45575</v>
       </c>
       <c r="H144" s="25" t="n">
-        <v>46993</v>
+        <v>47036</v>
       </c>
       <c r="I144" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="J144" t="n">
         <v>4</v>
@@ -23271,7 +23271,7 @@
         </is>
       </c>
       <c r="M144" s="25" t="n">
-        <v>46993</v>
+        <v>47036</v>
       </c>
       <c r="N144" t="n">
         <v>1</v>
@@ -23280,7 +23280,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>YM41D</t>
+          <t>YMCTD</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -23305,20 +23305,17 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t>AR0675705039</t>
+          <t>AR0688075032</t>
         </is>
       </c>
       <c r="G145" s="25" t="n">
-        <v>45938</v>
+        <v>45209</v>
       </c>
       <c r="H145" s="25" t="n">
-        <v>46395</v>
+        <v>46305</v>
       </c>
       <c r="I145" t="n">
-        <v>6</v>
-      </c>
-      <c r="J145" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K145" t="inlineStr">
         <is>
@@ -23331,16 +23328,22 @@
         </is>
       </c>
       <c r="M145" s="25" t="n">
-        <v>46395</v>
+        <v>46305</v>
       </c>
       <c r="N145" t="n">
         <v>1</v>
       </c>
+      <c r="O145" t="n">
+        <v>1</v>
+      </c>
+      <c r="P145" t="n">
+        <v>17.5</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>YMCYD</t>
+          <t>YM37D</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -23365,17 +23368,17 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>AR0417757066</t>
+          <t>AR0657794191</t>
         </is>
       </c>
       <c r="G146" s="25" t="n">
-        <v>45575</v>
+        <v>45784</v>
       </c>
       <c r="H146" s="25" t="n">
-        <v>47036</v>
+        <v>46514</v>
       </c>
       <c r="I146" t="n">
-        <v>6.5</v>
+        <v>7</v>
       </c>
       <c r="J146" t="n">
         <v>4</v>
@@ -23391,7 +23394,7 @@
         </is>
       </c>
       <c r="M146" s="25" t="n">
-        <v>47036</v>
+        <v>46514</v>
       </c>
       <c r="N146" t="n">
         <v>1</v>
@@ -23400,7 +23403,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>YMCTD</t>
+          <t>YM35D</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -23425,17 +23428,20 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>AR0688075032</t>
+          <t>AR0929824099</t>
         </is>
       </c>
       <c r="G147" s="25" t="n">
-        <v>45209</v>
+        <v>45715</v>
       </c>
       <c r="H147" s="25" t="n">
-        <v>46305</v>
+        <v>46445</v>
       </c>
       <c r="I147" t="n">
-        <v>0</v>
+        <v>6.25</v>
+      </c>
+      <c r="J147" t="n">
+        <v>4</v>
       </c>
       <c r="K147" t="inlineStr">
         <is>
@@ -23448,22 +23454,16 @@
         </is>
       </c>
       <c r="M147" s="25" t="n">
-        <v>46305</v>
+        <v>46445</v>
       </c>
       <c r="N147" t="n">
         <v>1</v>
       </c>
-      <c r="O147" t="n">
-        <v>1</v>
-      </c>
-      <c r="P147" t="n">
-        <v>17.5</v>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>YM37D</t>
+          <t>YM39D</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -23488,20 +23488,20 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>AR0657794191</t>
+          <t>AR0081455617</t>
         </is>
       </c>
       <c r="G148" s="25" t="n">
-        <v>45784</v>
+        <v>45860</v>
       </c>
       <c r="H148" s="25" t="n">
-        <v>46514</v>
+        <v>47686</v>
       </c>
       <c r="I148" t="n">
-        <v>7</v>
+        <v>8.75</v>
       </c>
       <c r="J148" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K148" t="inlineStr">
         <is>
@@ -23514,7 +23514,7 @@
         </is>
       </c>
       <c r="M148" s="25" t="n">
-        <v>46514</v>
+        <v>47686</v>
       </c>
       <c r="N148" t="n">
         <v>1</v>
@@ -23523,7 +23523,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>YM35D</t>
+          <t>YM38D</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -23548,17 +23548,17 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>AR0929824099</t>
+          <t>AR0419238511</t>
         </is>
       </c>
       <c r="G149" s="25" t="n">
-        <v>45715</v>
+        <v>45860</v>
       </c>
       <c r="H149" s="25" t="n">
-        <v>46445</v>
+        <v>46590</v>
       </c>
       <c r="I149" t="n">
-        <v>6.25</v>
+        <v>7.5</v>
       </c>
       <c r="J149" t="n">
         <v>4</v>
@@ -23574,7 +23574,7 @@
         </is>
       </c>
       <c r="M149" s="25" t="n">
-        <v>46445</v>
+        <v>46590</v>
       </c>
       <c r="N149" t="n">
         <v>1</v>
@@ -23583,7 +23583,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>YM39D</t>
+          <t>YM42D</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -23608,17 +23608,17 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>AR0081455617</t>
+          <t>AR0123407162</t>
         </is>
       </c>
       <c r="G150" s="25" t="n">
-        <v>45860</v>
+        <v>45993</v>
       </c>
       <c r="H150" s="25" t="n">
-        <v>47686</v>
+        <v>47179</v>
       </c>
       <c r="I150" t="n">
-        <v>8.75</v>
+        <v>7</v>
       </c>
       <c r="J150" t="n">
         <v>2</v>
@@ -23634,7 +23634,7 @@
         </is>
       </c>
       <c r="M150" s="25" t="n">
-        <v>47686</v>
+        <v>47179</v>
       </c>
       <c r="N150" t="n">
         <v>1</v>
@@ -23643,7 +23643,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>YM38D</t>
+          <t>YMCWD</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -23668,17 +23668,17 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>AR0419238511</t>
+          <t>AR0132676112</t>
         </is>
       </c>
       <c r="G151" s="25" t="n">
-        <v>45860</v>
+        <v>45474</v>
       </c>
       <c r="H151" s="25" t="n">
-        <v>46590</v>
+        <v>46204</v>
       </c>
       <c r="I151" t="n">
-        <v>7.5</v>
+        <v>1</v>
       </c>
       <c r="J151" t="n">
         <v>4</v>
@@ -23694,16 +23694,19 @@
         </is>
       </c>
       <c r="M151" s="25" t="n">
-        <v>46590</v>
+        <v>46204</v>
       </c>
       <c r="N151" t="n">
         <v>1</v>
       </c>
+      <c r="O151" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>YM42D</t>
+          <t>YMCRD</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -23728,20 +23731,20 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>AR0123407162</t>
+          <t>ARYPFS5601X8</t>
         </is>
       </c>
       <c r="G152" s="25" t="n">
-        <v>45993</v>
+        <v>45181</v>
       </c>
       <c r="H152" s="25" t="n">
-        <v>47179</v>
+        <v>47008</v>
       </c>
       <c r="I152" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="J152" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K152" t="inlineStr">
         <is>
@@ -23754,21 +23757,24 @@
         </is>
       </c>
       <c r="M152" s="25" t="n">
-        <v>47179</v>
+        <v>47008</v>
       </c>
       <c r="N152" t="n">
         <v>1</v>
       </c>
+      <c r="O152" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>YMCWD</t>
+          <t>IRCFD</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>YPF SA</t>
+          <t>IRSA S.A</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -23778,60 +23784,63 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Petróleo y Gas</t>
+          <t xml:space="preserve">Construcción </t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>NY</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>AR0132676112</t>
+          <t>USP58809BH95</t>
         </is>
       </c>
       <c r="G153" s="25" t="n">
-        <v>45474</v>
+        <v>44750</v>
       </c>
       <c r="H153" s="25" t="n">
-        <v>46204</v>
+        <v>46926</v>
       </c>
       <c r="I153" t="n">
-        <v>1</v>
+        <v>8.75</v>
       </c>
       <c r="J153" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>ACT/365</t>
+          <t>30/360</t>
         </is>
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>bullet</t>
+          <t>amortizing</t>
         </is>
       </c>
       <c r="M153" s="25" t="n">
-        <v>46204</v>
+        <v>45465</v>
       </c>
       <c r="N153" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="O153" t="n">
         <v>1</v>
       </c>
+      <c r="P153" t="n">
+        <v>17.5</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>YMCRD</t>
+          <t>TLCPD</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>YPF SA</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -23841,7 +23850,7 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Petróleo y Gas</t>
+          <t>Telecomunicaciones</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
@@ -23851,50 +23860,53 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t>ARYPFS5601X8</t>
+          <t>USP9028NCA74</t>
         </is>
       </c>
       <c r="G154" s="25" t="n">
-        <v>45181</v>
+        <v>45805</v>
       </c>
       <c r="H154" s="25" t="n">
-        <v>47008</v>
+        <v>48727</v>
       </c>
       <c r="I154" t="n">
-        <v>0</v>
+        <v>9.25</v>
       </c>
       <c r="J154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>ACT/365</t>
+          <t>30/360</t>
         </is>
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>bullet</t>
+          <t>amortizing</t>
         </is>
       </c>
       <c r="M154" s="25" t="n">
-        <v>47008</v>
+        <v>48362</v>
       </c>
       <c r="N154" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O154" t="n">
         <v>1</v>
       </c>
+      <c r="P154" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>IRCFD</t>
+          <t>TLCTD</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>IRSA S.A</t>
+          <t>Telecom</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -23904,7 +23916,7 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Construcción </t>
+          <t>Telecomunicaciones</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
@@ -23914,17 +23926,17 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>USP58809BH95</t>
+          <t>USP9028NCE96</t>
         </is>
       </c>
       <c r="G155" s="25" t="n">
-        <v>44750</v>
+        <v>46042</v>
       </c>
       <c r="H155" s="25" t="n">
-        <v>46926</v>
+        <v>49694</v>
       </c>
       <c r="I155" t="n">
-        <v>8.75</v>
+        <v>8.5</v>
       </c>
       <c r="J155" t="n">
         <v>2</v>
@@ -23940,27 +23952,27 @@
         </is>
       </c>
       <c r="M155" s="25" t="n">
-        <v>45465</v>
+        <v>49329</v>
       </c>
       <c r="N155" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="O155" t="n">
         <v>1</v>
       </c>
       <c r="P155" t="n">
-        <v>17.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TLCPD</t>
+          <t>YFCID</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>YPF Energia Electrica SA</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -23970,7 +23982,7 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Telecomunicaciones</t>
+          <t>Servicios Públicos y Generación</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
@@ -23980,20 +23992,20 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>USP9028NCA74</t>
+          <t>AR0947502206</t>
         </is>
       </c>
       <c r="G156" s="25" t="n">
-        <v>45805</v>
+        <v>45456</v>
       </c>
       <c r="H156" s="25" t="n">
-        <v>48727</v>
+        <v>46551</v>
       </c>
       <c r="I156" t="n">
-        <v>9.25</v>
+        <v>5.9</v>
       </c>
       <c r="J156" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K156" t="inlineStr">
         <is>
@@ -24006,13 +24018,13 @@
         </is>
       </c>
       <c r="M156" s="25" t="n">
-        <v>48362</v>
+        <v>46520</v>
       </c>
       <c r="N156" t="n">
         <v>2</v>
       </c>
       <c r="O156" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P156" t="n">
         <v>0</v>
@@ -24021,12 +24033,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>TLCTD</t>
+          <t>YM43D</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Telecom</t>
+          <t>YPF SA</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -24036,184 +24048,108 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Telecomunicaciones</t>
+          <t>Petróleo y Gas</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>NY</t>
+          <t>AR</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>USP9028NCE96</t>
+          <t>AR0156884063</t>
         </is>
       </c>
       <c r="G157" s="25" t="n">
-        <v>46042</v>
+        <v>46126</v>
       </c>
       <c r="H157" s="25" t="n">
-        <v>49694</v>
+        <v>47587</v>
       </c>
       <c r="I157" t="n">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="J157" t="n">
         <v>2</v>
       </c>
       <c r="K157" t="inlineStr">
         <is>
-          <t>30/360</t>
+          <t>ACT/365</t>
         </is>
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>amortizing</t>
+          <t>bullet</t>
         </is>
       </c>
       <c r="M157" s="25" t="n">
-        <v>49329</v>
+        <v>47588</v>
       </c>
       <c r="N157" t="n">
-        <v>2</v>
-      </c>
-      <c r="O157" t="n">
         <v>1</v>
       </c>
-      <c r="P157" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>YFCID</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>YPF Energia Electrica SA</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
+      <c r="A158" s="24" t="inlineStr">
+        <is>
+          <t>AERBD</t>
+        </is>
+      </c>
+      <c r="B158" s="24" t="n"/>
+      <c r="C158" s="24" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>Servicios Públicos y Generación</t>
-        </is>
-      </c>
-      <c r="E158" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>AR0947502206</t>
-        </is>
-      </c>
-      <c r="G158" s="25" t="n">
-        <v>45456</v>
-      </c>
-      <c r="H158" s="25" t="n">
-        <v>46551</v>
-      </c>
-      <c r="I158" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="J158" t="n">
-        <v>4</v>
-      </c>
-      <c r="K158" t="inlineStr">
-        <is>
-          <t>30/360</t>
-        </is>
-      </c>
-      <c r="L158" t="inlineStr">
-        <is>
-          <t>amortizing</t>
-        </is>
-      </c>
-      <c r="M158" s="25" t="n">
-        <v>46520</v>
-      </c>
-      <c r="N158" t="n">
-        <v>2</v>
-      </c>
-      <c r="O158" t="n">
-        <v>2</v>
-      </c>
-      <c r="P158" t="n">
-        <v>0</v>
-      </c>
+      <c r="D158" s="24" t="n"/>
+      <c r="E158" s="24" t="n"/>
+      <c r="F158" s="24" t="n"/>
+      <c r="G158" s="24" t="n"/>
+      <c r="H158" s="24" t="n"/>
+      <c r="I158" s="24" t="n"/>
+      <c r="J158" s="24" t="n"/>
+      <c r="K158" s="24" t="n"/>
+      <c r="L158" s="24" t="n"/>
+      <c r="M158" s="24" t="n"/>
+      <c r="N158" s="24" t="n"/>
+      <c r="O158" s="24" t="n"/>
+      <c r="P158" s="24" t="n"/>
+      <c r="Q158" s="24" t="n"/>
+      <c r="R158" s="24" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>YM43D</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>YPF SA</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
+      <c r="A159" s="24" t="inlineStr">
+        <is>
+          <t>AFCHD</t>
+        </is>
+      </c>
+      <c r="B159" s="24" t="n"/>
+      <c r="C159" s="24" t="inlineStr">
         <is>
           <t>ON</t>
         </is>
       </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>Petróleo y Gas</t>
-        </is>
-      </c>
-      <c r="E159" t="inlineStr">
-        <is>
-          <t>AR</t>
-        </is>
-      </c>
-      <c r="F159" t="inlineStr">
-        <is>
-          <t>AR0156884063</t>
-        </is>
-      </c>
-      <c r="G159" s="25" t="n">
-        <v>46126</v>
-      </c>
-      <c r="H159" s="25" t="n">
-        <v>47587</v>
-      </c>
-      <c r="I159" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="J159" t="n">
-        <v>2</v>
-      </c>
-      <c r="K159" t="inlineStr">
-        <is>
-          <t>ACT/365</t>
-        </is>
-      </c>
-      <c r="L159" t="inlineStr">
-        <is>
-          <t>bullet</t>
-        </is>
-      </c>
-      <c r="M159" s="25" t="n">
-        <v>47588</v>
-      </c>
-      <c r="N159" t="n">
-        <v>1</v>
-      </c>
+      <c r="D159" s="24" t="n"/>
+      <c r="E159" s="24" t="n"/>
+      <c r="F159" s="24" t="n"/>
+      <c r="G159" s="24" t="n"/>
+      <c r="H159" s="24" t="n"/>
+      <c r="I159" s="24" t="n"/>
+      <c r="J159" s="24" t="n"/>
+      <c r="K159" s="24" t="n"/>
+      <c r="L159" s="24" t="n"/>
+      <c r="M159" s="24" t="n"/>
+      <c r="N159" s="24" t="n"/>
+      <c r="O159" s="24" t="n"/>
+      <c r="P159" s="24" t="n"/>
+      <c r="Q159" s="24" t="n"/>
+      <c r="R159" s="24" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="24" t="inlineStr">
         <is>
-          <t>AERBD</t>
+          <t>AFCID</t>
         </is>
       </c>
       <c r="B160" s="24" t="n"/>
@@ -24241,7 +24177,7 @@
     <row r="161">
       <c r="A161" s="24" t="inlineStr">
         <is>
-          <t>AFCHD</t>
+          <t>AFCJD</t>
         </is>
       </c>
       <c r="B161" s="24" t="n"/>
@@ -24269,7 +24205,7 @@
     <row r="162">
       <c r="A162" s="24" t="inlineStr">
         <is>
-          <t>AFCID</t>
+          <t>AFCKD</t>
         </is>
       </c>
       <c r="B162" s="24" t="n"/>
@@ -24297,7 +24233,7 @@
     <row r="163">
       <c r="A163" s="24" t="inlineStr">
         <is>
-          <t>AFCJD</t>
+          <t>BACHD</t>
         </is>
       </c>
       <c r="B163" s="24" t="n"/>
@@ -24325,7 +24261,7 @@
     <row r="164">
       <c r="A164" s="24" t="inlineStr">
         <is>
-          <t>AFCKD</t>
+          <t>BF37D</t>
         </is>
       </c>
       <c r="B164" s="24" t="n"/>
@@ -24353,7 +24289,7 @@
     <row r="165">
       <c r="A165" s="24" t="inlineStr">
         <is>
-          <t>BACHD</t>
+          <t>BF40D</t>
         </is>
       </c>
       <c r="B165" s="24" t="n"/>
@@ -24381,7 +24317,7 @@
     <row r="166">
       <c r="A166" s="24" t="inlineStr">
         <is>
-          <t>BF37D</t>
+          <t>BF45D</t>
         </is>
       </c>
       <c r="B166" s="24" t="n"/>
@@ -24409,7 +24345,7 @@
     <row r="167">
       <c r="A167" s="24" t="inlineStr">
         <is>
-          <t>BF40D</t>
+          <t>BGC4D</t>
         </is>
       </c>
       <c r="B167" s="24" t="n"/>
@@ -24437,7 +24373,7 @@
     <row r="168">
       <c r="A168" s="24" t="inlineStr">
         <is>
-          <t>BF45D</t>
+          <t>BPCSD</t>
         </is>
       </c>
       <c r="B168" s="24" t="n"/>
@@ -24465,7 +24401,7 @@
     <row r="169">
       <c r="A169" s="24" t="inlineStr">
         <is>
-          <t>BGC4D</t>
+          <t>BPCUD</t>
         </is>
       </c>
       <c r="B169" s="24" t="n"/>
@@ -24493,7 +24429,7 @@
     <row r="170">
       <c r="A170" s="24" t="inlineStr">
         <is>
-          <t>BPCSD</t>
+          <t>BPCVD</t>
         </is>
       </c>
       <c r="B170" s="24" t="n"/>
@@ -24521,7 +24457,7 @@
     <row r="171">
       <c r="A171" s="24" t="inlineStr">
         <is>
-          <t>BPCUD</t>
+          <t>BVCPD</t>
         </is>
       </c>
       <c r="B171" s="24" t="n"/>
@@ -24549,7 +24485,7 @@
     <row r="172">
       <c r="A172" s="24" t="inlineStr">
         <is>
-          <t>BPCVD</t>
+          <t>CACBD</t>
         </is>
       </c>
       <c r="B172" s="24" t="n"/>
@@ -24577,7 +24513,7 @@
     <row r="173">
       <c r="A173" s="24" t="inlineStr">
         <is>
-          <t>BVCPD</t>
+          <t>CIC7D</t>
         </is>
       </c>
       <c r="B173" s="24" t="n"/>
@@ -24605,7 +24541,7 @@
     <row r="174">
       <c r="A174" s="24" t="inlineStr">
         <is>
-          <t>CACBD</t>
+          <t>CIC8D</t>
         </is>
       </c>
       <c r="B174" s="24" t="n"/>
@@ -24633,7 +24569,7 @@
     <row r="175">
       <c r="A175" s="24" t="inlineStr">
         <is>
-          <t>CIC7D</t>
+          <t>CIC9D</t>
         </is>
       </c>
       <c r="B175" s="24" t="n"/>
@@ -24661,7 +24597,7 @@
     <row r="176">
       <c r="A176" s="24" t="inlineStr">
         <is>
-          <t>CIC8D</t>
+          <t>CICBD</t>
         </is>
       </c>
       <c r="B176" s="24" t="n"/>
@@ -24689,7 +24625,7 @@
     <row r="177">
       <c r="A177" s="24" t="inlineStr">
         <is>
-          <t>CIC9D</t>
+          <t>CLI1D</t>
         </is>
       </c>
       <c r="B177" s="24" t="n"/>
@@ -24717,7 +24653,7 @@
     <row r="178">
       <c r="A178" s="24" t="inlineStr">
         <is>
-          <t>CICBD</t>
+          <t>CLSID</t>
         </is>
       </c>
       <c r="B178" s="24" t="n"/>
@@ -24745,7 +24681,7 @@
     <row r="179">
       <c r="A179" s="24" t="inlineStr">
         <is>
-          <t>CLI1D</t>
+          <t>CP37D</t>
         </is>
       </c>
       <c r="B179" s="24" t="n"/>
@@ -24773,7 +24709,7 @@
     <row r="180">
       <c r="A180" s="24" t="inlineStr">
         <is>
-          <t>CLSID</t>
+          <t>CP38D</t>
         </is>
       </c>
       <c r="B180" s="24" t="n"/>
@@ -24801,7 +24737,7 @@
     <row r="181">
       <c r="A181" s="24" t="inlineStr">
         <is>
-          <t>CP37D</t>
+          <t>CS45D</t>
         </is>
       </c>
       <c r="B181" s="24" t="n"/>
@@ -24829,7 +24765,7 @@
     <row r="182">
       <c r="A182" s="24" t="inlineStr">
         <is>
-          <t>CP38D</t>
+          <t>CS51D</t>
         </is>
       </c>
       <c r="B182" s="24" t="n"/>
@@ -24857,7 +24793,7 @@
     <row r="183">
       <c r="A183" s="24" t="inlineStr">
         <is>
-          <t>CS45D</t>
+          <t>CS52D</t>
         </is>
       </c>
       <c r="B183" s="24" t="n"/>
@@ -24885,7 +24821,7 @@
     <row r="184">
       <c r="A184" s="24" t="inlineStr">
         <is>
-          <t>CS51D</t>
+          <t>CWC6D</t>
         </is>
       </c>
       <c r="B184" s="24" t="n"/>
@@ -24913,7 +24849,7 @@
     <row r="185">
       <c r="A185" s="24" t="inlineStr">
         <is>
-          <t>CS52D</t>
+          <t>DEC2D</t>
         </is>
       </c>
       <c r="B185" s="24" t="n"/>
@@ -24941,7 +24877,7 @@
     <row r="186">
       <c r="A186" s="24" t="inlineStr">
         <is>
-          <t>CWC6D</t>
+          <t>DNCAD</t>
         </is>
       </c>
       <c r="B186" s="24" t="n"/>
@@ -24969,7 +24905,7 @@
     <row r="187">
       <c r="A187" s="24" t="inlineStr">
         <is>
-          <t>DEC2D</t>
+          <t>EAC3D</t>
         </is>
       </c>
       <c r="B187" s="24" t="n"/>
@@ -24997,7 +24933,7 @@
     <row r="188">
       <c r="A188" s="24" t="inlineStr">
         <is>
-          <t>DNCAD</t>
+          <t>FO4AD</t>
         </is>
       </c>
       <c r="B188" s="24" t="n"/>
@@ -25025,7 +24961,7 @@
     <row r="189">
       <c r="A189" s="24" t="inlineStr">
         <is>
-          <t>EAC3D</t>
+          <t>FYC1D</t>
         </is>
       </c>
       <c r="B189" s="24" t="n"/>
@@ -25053,7 +24989,7 @@
     <row r="190">
       <c r="A190" s="24" t="inlineStr">
         <is>
-          <t>FO4AD</t>
+          <t>GN43D</t>
         </is>
       </c>
       <c r="B190" s="24" t="n"/>
@@ -25081,7 +25017,7 @@
     <row r="191">
       <c r="A191" s="24" t="inlineStr">
         <is>
-          <t>FYC1D</t>
+          <t>GN47D</t>
         </is>
       </c>
       <c r="B191" s="24" t="n"/>
@@ -25109,7 +25045,7 @@
     <row r="192">
       <c r="A192" s="24" t="inlineStr">
         <is>
-          <t>GN43D</t>
+          <t>GN48D</t>
         </is>
       </c>
       <c r="B192" s="24" t="n"/>
@@ -25137,7 +25073,7 @@
     <row r="193">
       <c r="A193" s="24" t="inlineStr">
         <is>
-          <t>GN47D</t>
+          <t>GN49D</t>
         </is>
       </c>
       <c r="B193" s="24" t="n"/>
@@ -25165,7 +25101,7 @@
     <row r="194">
       <c r="A194" s="24" t="inlineStr">
         <is>
-          <t>GN48D</t>
+          <t>GOC4D</t>
         </is>
       </c>
       <c r="B194" s="24" t="n"/>
@@ -25193,7 +25129,7 @@
     <row r="195">
       <c r="A195" s="24" t="inlineStr">
         <is>
-          <t>GN49D</t>
+          <t>GYC4D</t>
         </is>
       </c>
       <c r="B195" s="24" t="n"/>
@@ -25221,7 +25157,7 @@
     <row r="196">
       <c r="A196" s="24" t="inlineStr">
         <is>
-          <t>GOC4D</t>
+          <t>GYC5D</t>
         </is>
       </c>
       <c r="B196" s="24" t="n"/>
@@ -25249,7 +25185,7 @@
     <row r="197">
       <c r="A197" s="24" t="inlineStr">
         <is>
-          <t>GYC4D</t>
+          <t>HBCAD</t>
         </is>
       </c>
       <c r="B197" s="24" t="n"/>
@@ -25277,7 +25213,7 @@
     <row r="198">
       <c r="A198" s="24" t="inlineStr">
         <is>
-          <t>GYC5D</t>
+          <t>HBCDD</t>
         </is>
       </c>
       <c r="B198" s="24" t="n"/>
@@ -25305,7 +25241,7 @@
     <row r="199">
       <c r="A199" s="24" t="inlineStr">
         <is>
-          <t>HBCAD</t>
+          <t>HJCFD</t>
         </is>
       </c>
       <c r="B199" s="24" t="n"/>
@@ -25333,7 +25269,7 @@
     <row r="200">
       <c r="A200" s="24" t="inlineStr">
         <is>
-          <t>HBCDD</t>
+          <t>HJCGD</t>
         </is>
       </c>
       <c r="B200" s="24" t="n"/>
@@ -25361,7 +25297,7 @@
     <row r="201">
       <c r="A201" s="24" t="inlineStr">
         <is>
-          <t>HJCFD</t>
+          <t>HVS1D</t>
         </is>
       </c>
       <c r="B201" s="24" t="n"/>
@@ -25389,7 +25325,7 @@
     <row r="202">
       <c r="A202" s="24" t="inlineStr">
         <is>
-          <t>HJCGD</t>
+          <t>JNC5D</t>
         </is>
       </c>
       <c r="B202" s="24" t="n"/>
@@ -25417,7 +25353,7 @@
     <row r="203">
       <c r="A203" s="24" t="inlineStr">
         <is>
-          <t>HVS1D</t>
+          <t>JNC6D</t>
         </is>
       </c>
       <c r="B203" s="24" t="n"/>
@@ -25445,7 +25381,7 @@
     <row r="204">
       <c r="A204" s="24" t="inlineStr">
         <is>
-          <t>JNC5D</t>
+          <t>LDCGD</t>
         </is>
       </c>
       <c r="B204" s="24" t="n"/>
@@ -25473,7 +25409,7 @@
     <row r="205">
       <c r="A205" s="24" t="inlineStr">
         <is>
-          <t>JNC6D</t>
+          <t>LIC6D</t>
         </is>
       </c>
       <c r="B205" s="24" t="n"/>
@@ -25501,7 +25437,7 @@
     <row r="206">
       <c r="A206" s="24" t="inlineStr">
         <is>
-          <t>LDCGD</t>
+          <t>LUC5D</t>
         </is>
       </c>
       <c r="B206" s="24" t="n"/>
@@ -25529,7 +25465,7 @@
     <row r="207">
       <c r="A207" s="24" t="inlineStr">
         <is>
-          <t>LIC6D</t>
+          <t>MCC1D</t>
         </is>
       </c>
       <c r="B207" s="24" t="n"/>
@@ -25557,7 +25493,7 @@
     <row r="208">
       <c r="A208" s="24" t="inlineStr">
         <is>
-          <t>LUC5D</t>
+          <t>MCC2D</t>
         </is>
       </c>
       <c r="B208" s="24" t="n"/>
@@ -25585,7 +25521,7 @@
     <row r="209">
       <c r="A209" s="24" t="inlineStr">
         <is>
-          <t>MCC1D</t>
+          <t>MCC3D</t>
         </is>
       </c>
       <c r="B209" s="24" t="n"/>
@@ -25613,7 +25549,7 @@
     <row r="210">
       <c r="A210" s="24" t="inlineStr">
         <is>
-          <t>MCC2D</t>
+          <t>MIC3D</t>
         </is>
       </c>
       <c r="B210" s="24" t="n"/>
@@ -25641,7 +25577,7 @@
     <row r="211">
       <c r="A211" s="24" t="inlineStr">
         <is>
-          <t>MCC3D</t>
+          <t>MIC4D</t>
         </is>
       </c>
       <c r="B211" s="24" t="n"/>
@@ -25669,7 +25605,7 @@
     <row r="212">
       <c r="A212" s="24" t="inlineStr">
         <is>
-          <t>MIC3D</t>
+          <t>MIC6D</t>
         </is>
       </c>
       <c r="B212" s="24" t="n"/>
@@ -25697,7 +25633,7 @@
     <row r="213">
       <c r="A213" s="24" t="inlineStr">
         <is>
-          <t>MIC4D</t>
+          <t>MR39D</t>
         </is>
       </c>
       <c r="B213" s="24" t="n"/>
@@ -25725,7 +25661,7 @@
     <row r="214">
       <c r="A214" s="24" t="inlineStr">
         <is>
-          <t>MIC6D</t>
+          <t>MSSED</t>
         </is>
       </c>
       <c r="B214" s="24" t="n"/>
@@ -25753,7 +25689,7 @@
     <row r="215">
       <c r="A215" s="24" t="inlineStr">
         <is>
-          <t>MR39D</t>
+          <t>MSSFD</t>
         </is>
       </c>
       <c r="B215" s="24" t="n"/>
@@ -25781,7 +25717,7 @@
     <row r="216">
       <c r="A216" s="24" t="inlineStr">
         <is>
-          <t>MSSED</t>
+          <t>MSSGD</t>
         </is>
       </c>
       <c r="B216" s="24" t="n"/>
@@ -25809,7 +25745,7 @@
     <row r="217">
       <c r="A217" s="24" t="inlineStr">
         <is>
-          <t>MSSFD</t>
+          <t>MU31D</t>
         </is>
       </c>
       <c r="B217" s="24" t="n"/>
@@ -25837,7 +25773,7 @@
     <row r="218">
       <c r="A218" s="24" t="inlineStr">
         <is>
-          <t>MSSGD</t>
+          <t>MU32D</t>
         </is>
       </c>
       <c r="B218" s="24" t="n"/>
@@ -25865,7 +25801,7 @@
     <row r="219">
       <c r="A219" s="24" t="inlineStr">
         <is>
-          <t>MU31D</t>
+          <t>NBS1D</t>
         </is>
       </c>
       <c r="B219" s="24" t="n"/>
@@ -25893,7 +25829,7 @@
     <row r="220">
       <c r="A220" s="24" t="inlineStr">
         <is>
-          <t>MU32D</t>
+          <t>NPCDD</t>
         </is>
       </c>
       <c r="B220" s="24" t="n"/>
@@ -25921,7 +25857,7 @@
     <row r="221">
       <c r="A221" s="24" t="inlineStr">
         <is>
-          <t>NBS1D</t>
+          <t>OT41D</t>
         </is>
       </c>
       <c r="B221" s="24" t="n"/>
@@ -25949,7 +25885,7 @@
     <row r="222">
       <c r="A222" s="24" t="inlineStr">
         <is>
-          <t>NPCDD</t>
+          <t>OZC3D</t>
         </is>
       </c>
       <c r="B222" s="24" t="n"/>
@@ -25977,7 +25913,7 @@
     <row r="223">
       <c r="A223" s="24" t="inlineStr">
         <is>
-          <t>OT41D</t>
+          <t>PECMD</t>
         </is>
       </c>
       <c r="B223" s="24" t="n"/>
@@ -26005,7 +25941,7 @@
     <row r="224">
       <c r="A224" s="24" t="inlineStr">
         <is>
-          <t>OZC3D</t>
+          <t>PECND</t>
         </is>
       </c>
       <c r="B224" s="24" t="n"/>
@@ -26033,7 +25969,7 @@
     <row r="225">
       <c r="A225" s="24" t="inlineStr">
         <is>
-          <t>PECMD</t>
+          <t>PFC3D</t>
         </is>
       </c>
       <c r="B225" s="24" t="n"/>
@@ -26061,7 +25997,7 @@
     <row r="226">
       <c r="A226" s="24" t="inlineStr">
         <is>
-          <t>PECND</t>
+          <t>PN34D</t>
         </is>
       </c>
       <c r="B226" s="24" t="n"/>
@@ -26089,7 +26025,7 @@
     <row r="227">
       <c r="A227" s="24" t="inlineStr">
         <is>
-          <t>PFC3D</t>
+          <t>PQCRD</t>
         </is>
       </c>
       <c r="B227" s="24" t="n"/>
@@ -26117,7 +26053,7 @@
     <row r="228">
       <c r="A228" s="24" t="inlineStr">
         <is>
-          <t>PN34D</t>
+          <t>PQCTD</t>
         </is>
       </c>
       <c r="B228" s="24" t="n"/>
@@ -26145,7 +26081,7 @@
     <row r="229">
       <c r="A229" s="24" t="inlineStr">
         <is>
-          <t>PQCRD</t>
+          <t>PZCGD</t>
         </is>
       </c>
       <c r="B229" s="24" t="n"/>
@@ -26173,7 +26109,7 @@
     <row r="230">
       <c r="A230" s="24" t="inlineStr">
         <is>
-          <t>PQCTD</t>
+          <t>RC1CD</t>
         </is>
       </c>
       <c r="B230" s="24" t="n"/>
@@ -26201,7 +26137,7 @@
     <row r="231">
       <c r="A231" s="24" t="inlineStr">
         <is>
-          <t>PZCGD</t>
+          <t>RC3CD</t>
         </is>
       </c>
       <c r="B231" s="24" t="n"/>
@@ -26229,7 +26165,7 @@
     <row r="232">
       <c r="A232" s="24" t="inlineStr">
         <is>
-          <t>RC1CD</t>
+          <t>RC5CD</t>
         </is>
       </c>
       <c r="B232" s="24" t="n"/>
@@ -26257,7 +26193,7 @@
     <row r="233">
       <c r="A233" s="24" t="inlineStr">
         <is>
-          <t>RC3CD</t>
+          <t>RZ9BD</t>
         </is>
       </c>
       <c r="B233" s="24" t="n"/>
@@ -26285,7 +26221,7 @@
     <row r="234">
       <c r="A234" s="24" t="inlineStr">
         <is>
-          <t>RC5CD</t>
+          <t>RZABD</t>
         </is>
       </c>
       <c r="B234" s="24" t="n"/>
@@ -26313,7 +26249,7 @@
     <row r="235">
       <c r="A235" s="24" t="inlineStr">
         <is>
-          <t>RZ9BD</t>
+          <t>SBC1D</t>
         </is>
       </c>
       <c r="B235" s="24" t="n"/>
@@ -26341,7 +26277,7 @@
     <row r="236">
       <c r="A236" s="24" t="inlineStr">
         <is>
-          <t>RZABD</t>
+          <t>SBC2D</t>
         </is>
       </c>
       <c r="B236" s="24" t="n"/>
@@ -26369,7 +26305,7 @@
     <row r="237">
       <c r="A237" s="24" t="inlineStr">
         <is>
-          <t>SBC1D</t>
+          <t>SIC1D</t>
         </is>
       </c>
       <c r="B237" s="24" t="n"/>
@@ -26397,7 +26333,7 @@
     <row r="238">
       <c r="A238" s="24" t="inlineStr">
         <is>
-          <t>SBC2D</t>
+          <t>SNABD</t>
         </is>
       </c>
       <c r="B238" s="24" t="n"/>
@@ -26425,7 +26361,7 @@
     <row r="239">
       <c r="A239" s="24" t="inlineStr">
         <is>
-          <t>SIC1D</t>
+          <t>SNEAD</t>
         </is>
       </c>
       <c r="B239" s="24" t="n"/>
@@ -26453,7 +26389,7 @@
     <row r="240">
       <c r="A240" s="24" t="inlineStr">
         <is>
-          <t>SNABD</t>
+          <t>SNEBD</t>
         </is>
       </c>
       <c r="B240" s="24" t="n"/>
@@ -26481,7 +26417,7 @@
     <row r="241">
       <c r="A241" s="24" t="inlineStr">
         <is>
-          <t>SNEAD</t>
+          <t>SNSBD</t>
         </is>
       </c>
       <c r="B241" s="24" t="n"/>
@@ -26509,7 +26445,7 @@
     <row r="242">
       <c r="A242" s="24" t="inlineStr">
         <is>
-          <t>SNEBD</t>
+          <t>SNSDD</t>
         </is>
       </c>
       <c r="B242" s="24" t="n"/>
@@ -26537,7 +26473,7 @@
     <row r="243">
       <c r="A243" s="24" t="inlineStr">
         <is>
-          <t>SNSBD</t>
+          <t>STCFD</t>
         </is>
       </c>
       <c r="B243" s="24" t="n"/>
@@ -26565,7 +26501,7 @@
     <row r="244">
       <c r="A244" s="24" t="inlineStr">
         <is>
-          <t>SNSDD</t>
+          <t>SXC4D</t>
         </is>
       </c>
       <c r="B244" s="24" t="n"/>
@@ -26593,7 +26529,7 @@
     <row r="245">
       <c r="A245" s="24" t="inlineStr">
         <is>
-          <t>STCFD</t>
+          <t>T641D</t>
         </is>
       </c>
       <c r="B245" s="24" t="n"/>
@@ -26621,7 +26557,7 @@
     <row r="246">
       <c r="A246" s="24" t="inlineStr">
         <is>
-          <t>SXC4D</t>
+          <t>T672D</t>
         </is>
       </c>
       <c r="B246" s="24" t="n"/>
@@ -26649,7 +26585,7 @@
     <row r="247">
       <c r="A247" s="24" t="inlineStr">
         <is>
-          <t>T641D</t>
+          <t>TLCVD</t>
         </is>
       </c>
       <c r="B247" s="24" t="n"/>
@@ -26677,7 +26613,7 @@
     <row r="248">
       <c r="A248" s="24" t="inlineStr">
         <is>
-          <t>T672D</t>
+          <t>TLCWD</t>
         </is>
       </c>
       <c r="B248" s="24" t="n"/>
@@ -26705,7 +26641,7 @@
     <row r="249">
       <c r="A249" s="24" t="inlineStr">
         <is>
-          <t>TLCVD</t>
+          <t>TTCED</t>
         </is>
       </c>
       <c r="B249" s="24" t="n"/>
@@ -26733,7 +26669,7 @@
     <row r="250">
       <c r="A250" s="24" t="inlineStr">
         <is>
-          <t>TLCWD</t>
+          <t>VBC1D</t>
         </is>
       </c>
       <c r="B250" s="24" t="n"/>
@@ -26761,7 +26697,7 @@
     <row r="251">
       <c r="A251" s="24" t="inlineStr">
         <is>
-          <t>TTCED</t>
+          <t>VBC2D</t>
         </is>
       </c>
       <c r="B251" s="24" t="n"/>
@@ -26789,7 +26725,7 @@
     <row r="252">
       <c r="A252" s="24" t="inlineStr">
         <is>
-          <t>VBC1D</t>
+          <t>VSCID</t>
         </is>
       </c>
       <c r="B252" s="24" t="n"/>
@@ -26817,7 +26753,7 @@
     <row r="253">
       <c r="A253" s="24" t="inlineStr">
         <is>
-          <t>VBC2D</t>
+          <t>VSCPD</t>
         </is>
       </c>
       <c r="B253" s="24" t="n"/>
@@ -26845,7 +26781,7 @@
     <row r="254">
       <c r="A254" s="24" t="inlineStr">
         <is>
-          <t>VSCID</t>
+          <t>VSCXD</t>
         </is>
       </c>
       <c r="B254" s="24" t="n"/>
@@ -26873,7 +26809,7 @@
     <row r="255">
       <c r="A255" s="24" t="inlineStr">
         <is>
-          <t>VSCPD</t>
+          <t>WBS1D</t>
         </is>
       </c>
       <c r="B255" s="24" t="n"/>
@@ -26901,7 +26837,7 @@
     <row r="256">
       <c r="A256" s="24" t="inlineStr">
         <is>
-          <t>VSCXD</t>
+          <t>YFCKD</t>
         </is>
       </c>
       <c r="B256" s="24" t="n"/>
@@ -26929,7 +26865,7 @@
     <row r="257">
       <c r="A257" s="24" t="inlineStr">
         <is>
-          <t>WBS1D</t>
+          <t>ZPC2D</t>
         </is>
       </c>
       <c r="B257" s="24" t="n"/>
@@ -26957,7 +26893,7 @@
     <row r="258">
       <c r="A258" s="24" t="inlineStr">
         <is>
-          <t>YFCKD</t>
+          <t>ZPC3D</t>
         </is>
       </c>
       <c r="B258" s="24" t="n"/>
@@ -26985,7 +26921,7 @@
     <row r="259">
       <c r="A259" s="24" t="inlineStr">
         <is>
-          <t>ZPC2D</t>
+          <t>PUC2D</t>
         </is>
       </c>
       <c r="B259" s="24" t="n"/>
@@ -27013,7 +26949,7 @@
     <row r="260">
       <c r="A260" s="24" t="inlineStr">
         <is>
-          <t>ZPC3D</t>
+          <t>ICC6D</t>
         </is>
       </c>
       <c r="B260" s="24" t="n"/>
@@ -27038,62 +26974,6 @@
       <c r="Q260" s="24" t="n"/>
       <c r="R260" s="24" t="n"/>
     </row>
-    <row r="261">
-      <c r="A261" s="24" t="inlineStr">
-        <is>
-          <t>PUC2D</t>
-        </is>
-      </c>
-      <c r="B261" s="24" t="n"/>
-      <c r="C261" s="24" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="D261" s="24" t="n"/>
-      <c r="E261" s="24" t="n"/>
-      <c r="F261" s="24" t="n"/>
-      <c r="G261" s="24" t="n"/>
-      <c r="H261" s="24" t="n"/>
-      <c r="I261" s="24" t="n"/>
-      <c r="J261" s="24" t="n"/>
-      <c r="K261" s="24" t="n"/>
-      <c r="L261" s="24" t="n"/>
-      <c r="M261" s="24" t="n"/>
-      <c r="N261" s="24" t="n"/>
-      <c r="O261" s="24" t="n"/>
-      <c r="P261" s="24" t="n"/>
-      <c r="Q261" s="24" t="n"/>
-      <c r="R261" s="24" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="24" t="inlineStr">
-        <is>
-          <t>ICC6D</t>
-        </is>
-      </c>
-      <c r="B262" s="24" t="n"/>
-      <c r="C262" s="24" t="inlineStr">
-        <is>
-          <t>ON</t>
-        </is>
-      </c>
-      <c r="D262" s="24" t="n"/>
-      <c r="E262" s="24" t="n"/>
-      <c r="F262" s="24" t="n"/>
-      <c r="G262" s="24" t="n"/>
-      <c r="H262" s="24" t="n"/>
-      <c r="I262" s="24" t="n"/>
-      <c r="J262" s="24" t="n"/>
-      <c r="K262" s="24" t="n"/>
-      <c r="L262" s="24" t="n"/>
-      <c r="M262" s="24" t="n"/>
-      <c r="N262" s="24" t="n"/>
-      <c r="O262" s="24" t="n"/>
-      <c r="P262" s="24" t="n"/>
-      <c r="Q262" s="24" t="n"/>
-      <c r="R262" s="24" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
mejoras de dolar futuro
</commit_message>
<xml_diff>
--- a/data/instruments_master.xlsx
+++ b/data/instruments_master.xlsx
@@ -14399,7 +14399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R263"/>
+  <dimension ref="A1:R265"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26904,6 +26904,62 @@
       <c r="Q263" s="24" t="n"/>
       <c r="R263" s="24" t="n"/>
     </row>
+    <row r="264">
+      <c r="A264" s="24" t="inlineStr">
+        <is>
+          <t>BF44D</t>
+        </is>
+      </c>
+      <c r="B264" s="24" t="n"/>
+      <c r="C264" s="24" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D264" s="24" t="n"/>
+      <c r="E264" s="24" t="n"/>
+      <c r="F264" s="24" t="n"/>
+      <c r="G264" s="24" t="n"/>
+      <c r="H264" s="24" t="n"/>
+      <c r="I264" s="24" t="n"/>
+      <c r="J264" s="24" t="n"/>
+      <c r="K264" s="24" t="n"/>
+      <c r="L264" s="24" t="n"/>
+      <c r="M264" s="24" t="n"/>
+      <c r="N264" s="24" t="n"/>
+      <c r="O264" s="24" t="n"/>
+      <c r="P264" s="24" t="n"/>
+      <c r="Q264" s="24" t="n"/>
+      <c r="R264" s="24" t="n"/>
+    </row>
+    <row r="265">
+      <c r="A265" s="24" t="inlineStr">
+        <is>
+          <t>RZBAD</t>
+        </is>
+      </c>
+      <c r="B265" s="24" t="n"/>
+      <c r="C265" s="24" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D265" s="24" t="n"/>
+      <c r="E265" s="24" t="n"/>
+      <c r="F265" s="24" t="n"/>
+      <c r="G265" s="24" t="n"/>
+      <c r="H265" s="24" t="n"/>
+      <c r="I265" s="24" t="n"/>
+      <c r="J265" s="24" t="n"/>
+      <c r="K265" s="24" t="n"/>
+      <c r="L265" s="24" t="n"/>
+      <c r="M265" s="24" t="n"/>
+      <c r="N265" s="24" t="n"/>
+      <c r="O265" s="24" t="n"/>
+      <c r="P265" s="24" t="n"/>
+      <c r="Q265" s="24" t="n"/>
+      <c r="R265" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
formateo para captura de whatsapp
</commit_message>
<xml_diff>
--- a/data/instruments_master.xlsx
+++ b/data/instruments_master.xlsx
@@ -22960,7 +22960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R269"/>
+  <dimension ref="A1:R270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37659,6 +37659,34 @@
       <c r="Q269" s="24" t="n"/>
       <c r="R269" s="24" t="n"/>
     </row>
+    <row r="270">
+      <c r="A270" s="24" t="inlineStr">
+        <is>
+          <t>SIC2D</t>
+        </is>
+      </c>
+      <c r="B270" s="24" t="n"/>
+      <c r="C270" s="24" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D270" s="24" t="n"/>
+      <c r="E270" s="24" t="n"/>
+      <c r="F270" s="24" t="n"/>
+      <c r="G270" s="24" t="n"/>
+      <c r="H270" s="24" t="n"/>
+      <c r="I270" s="24" t="n"/>
+      <c r="J270" s="24" t="n"/>
+      <c r="K270" s="24" t="n"/>
+      <c r="L270" s="24" t="n"/>
+      <c r="M270" s="24" t="n"/>
+      <c r="N270" s="24" t="n"/>
+      <c r="O270" s="24" t="n"/>
+      <c r="P270" s="24" t="n"/>
+      <c r="Q270" s="24" t="n"/>
+      <c r="R270" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Monitor de canje + curva log de historico
</commit_message>
<xml_diff>
--- a/data/instruments_master.xlsx
+++ b/data/instruments_master.xlsx
@@ -22960,7 +22960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R272"/>
+  <dimension ref="A1:R273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -37743,6 +37743,34 @@
       <c r="Q272" s="24" t="n"/>
       <c r="R272" s="24" t="n"/>
     </row>
+    <row r="273">
+      <c r="A273" s="24" t="inlineStr">
+        <is>
+          <t>AFCPD</t>
+        </is>
+      </c>
+      <c r="B273" s="24" t="n"/>
+      <c r="C273" s="24" t="inlineStr">
+        <is>
+          <t>ON</t>
+        </is>
+      </c>
+      <c r="D273" s="24" t="n"/>
+      <c r="E273" s="24" t="n"/>
+      <c r="F273" s="24" t="n"/>
+      <c r="G273" s="24" t="n"/>
+      <c r="H273" s="24" t="n"/>
+      <c r="I273" s="24" t="n"/>
+      <c r="J273" s="24" t="n"/>
+      <c r="K273" s="24" t="n"/>
+      <c r="L273" s="24" t="n"/>
+      <c r="M273" s="24" t="n"/>
+      <c r="N273" s="24" t="n"/>
+      <c r="O273" s="24" t="n"/>
+      <c r="P273" s="24" t="n"/>
+      <c r="Q273" s="24" t="n"/>
+      <c r="R273" s="24" t="n"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>